<commit_message>
Fix phone tel: links and color bar seams in 2026 signatures
- Render Main/Direct/Mobile phone numbers as plain text. The tel: anchors
  were being rewritten as "[tel;digits]" next to the number in sent mail.
- Remove the invisible 1x4 spacer image from each color bar cell. Outlook
  ignores opacity, so the image rendered as a dark 1px seam between segments.
- Drop border-collapse on the bar table to avoid hairline gaps in Outlook.
- Regenerate all 2026 signatures from the script (includes new entries from
  the updated employee spreadsheet).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/employees_spsi.xlsx
+++ b/employees_spsi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jscheftic\SPSI Code\SPSI Signatures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB8AB29-59BA-42B1-AF16-D0560366432B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EEAD8F-71A1-44E3-BE86-A5234D237E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30675" yWindow="1050" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="170">
   <si>
     <t>Name</t>
   </si>
@@ -500,6 +500,39 @@
   </si>
   <si>
     <t>South Central Manager</t>
+  </si>
+  <si>
+    <t>logan Beaubien</t>
+  </si>
+  <si>
+    <t>lbeaubien@spsi.com</t>
+  </si>
+  <si>
+    <t>Sales Development Representative</t>
+  </si>
+  <si>
+    <t>Juan Tapia</t>
+  </si>
+  <si>
+    <t>Apprentice Service Tech</t>
+  </si>
+  <si>
+    <t>763-255-1019</t>
+  </si>
+  <si>
+    <t>763-255-1013</t>
+  </si>
+  <si>
+    <t>jtapia@spsi.com</t>
+  </si>
+  <si>
+    <t>Michael Schwend</t>
+  </si>
+  <si>
+    <t>Sales Representative</t>
+  </si>
+  <si>
+    <t>mschwend@spsi.com</t>
   </si>
 </sst>
 </file>
@@ -926,7 +959,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" customWidth="1"/>
@@ -1734,7 +1767,7 @@
       <c r="H27" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="4" t="s">
         <v>134</v>
       </c>
       <c r="J27" s="2"/>
@@ -1999,6 +2032,90 @@
       </c>
       <c r="I37" s="5" t="s">
         <v>157</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>159</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G38">
+        <v>1019</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="I38" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>162</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G39">
+        <v>1013</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>167</v>
+      </c>
+      <c r="B40" t="s">
+        <v>168</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I40" s="5" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2015,6 +2132,9 @@
     <hyperlink ref="I35" r:id="rId8" xr:uid="{809D9758-0FE4-4826-A9DB-D6860327E3A1}"/>
     <hyperlink ref="I36" r:id="rId9" xr:uid="{D253A6F8-193A-4864-868D-36CAFD4E39CE}"/>
     <hyperlink ref="I37" r:id="rId10" xr:uid="{648EABE6-7C55-467B-9A28-2D6546C6E22C}"/>
+    <hyperlink ref="I39" r:id="rId11" xr:uid="{E1F5EE58-6B82-4AA6-9B5A-339B807499CC}"/>
+    <hyperlink ref="I40" r:id="rId12" xr:uid="{ACAFB5FC-D389-4A9B-A2F5-AD7AC08AC7B6}"/>
+    <hyperlink ref="I27" r:id="rId13" xr:uid="{BCD92F00-024D-4C67-9955-80F24563D390}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>